<commit_message>
chore: update sync bat and latest data snapshot
</commit_message>
<xml_diff>
--- a/Locker/Keys Lock Tracker - 2026 1.xlsx
+++ b/Locker/Keys Lock Tracker - 2026 1.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://cbre-my.sharepoint.com/personal/satyabrata_mohanty1_cbre_com/Documents/Desktop/Trackers/Locker/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="342" documentId="11_F56D8C5A66DACF4247F893C0199D457268BC86FF" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{0669E165-B7FC-433A-91B0-D711E43EEF81}"/>
+  <xr:revisionPtr revIDLastSave="434" documentId="11_F56D8C5A66DACF4247F893C0199D457268BC86FF" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{5BF8A4FE-C257-420E-8D6F-2E6E38366AE8}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="19200" windowHeight="11280" firstSheet="1" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2348" uniqueCount="392">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2390" uniqueCount="394">
   <si>
     <t>📊 Executive Dashboard</t>
   </si>
@@ -831,6 +831,9 @@
     <t>MR - 101</t>
   </si>
   <si>
+    <t>Box No-15</t>
+  </si>
+  <si>
     <t>Common Asset</t>
   </si>
   <si>
@@ -844,6 +847,9 @@
   </si>
   <si>
     <t>MR - 106</t>
+  </si>
+  <si>
+    <t>Box NO-15</t>
   </si>
   <si>
     <t>MR - 107</t>
@@ -2543,7 +2549,7 @@
   <autoFilter ref="A7:P257" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}">
     <filterColumn colId="2">
       <filters>
-        <filter val="705"/>
+        <filter val="280"/>
         <filter val="(NonBlanks)"/>
       </filters>
     </filterColumn>
@@ -2988,7 +2994,7 @@
     <row r="8" spans="2:16" ht="27.95" customHeight="1">
       <c r="B8" s="65">
         <f>COUNTA(Table_Tracker[Lock No.])</f>
-        <v>244</v>
+        <v>245</v>
       </c>
       <c r="C8" s="69"/>
       <c r="D8" s="69"/>
@@ -3009,7 +3015,7 @@
       <c r="M8" s="15"/>
       <c r="N8" s="61">
         <f>COUNTIF(Table_Tracker[Lock Status], "Common Asset")</f>
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="O8" s="69"/>
       <c r="P8" s="69"/>
@@ -3067,14 +3073,14 @@
     <row r="12" spans="2:16" ht="27.95" customHeight="1">
       <c r="B12" s="55">
         <f>SUM(Table_Tracker[Total Keys])</f>
-        <v>529</v>
+        <v>531</v>
       </c>
       <c r="C12" s="69"/>
       <c r="D12" s="69"/>
       <c r="E12" s="15"/>
       <c r="F12" s="50">
         <f>SUM(Table_Tracker[Spare Keys (BMS)])</f>
-        <v>372</v>
+        <v>376</v>
       </c>
       <c r="G12" s="69"/>
       <c r="H12" s="69"/>
@@ -3088,7 +3094,7 @@
       <c r="M12" s="15"/>
       <c r="N12" s="52">
         <f>SUM(Table_Tracker[Missing Keys])</f>
-        <v>68</v>
+        <v>66</v>
       </c>
       <c r="O12" s="69"/>
       <c r="P12" s="69"/>
@@ -3275,7 +3281,7 @@
       </c>
       <c r="K18" s="5">
         <f>COUNTIF(Table_Tracker[Lock Type], "Cupboard")</f>
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="L18" s="5">
         <f>COUNTIFS(Table_Tracker[Lock Type], "Cupboard", Table_Tracker[Lock Status], "Occupied")</f>
@@ -3287,7 +3293,7 @@
       </c>
       <c r="N18" s="5">
         <f>SUMIFS(Table_Tracker[Spare Keys (BMS)], Table_Tracker[Lock Type], "Cupboard")</f>
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="O18" s="5">
         <f>SUMIFS(Table_Tracker[Issued Keys], Table_Tracker[Lock Type], "Cupboard")</f>
@@ -3304,7 +3310,7 @@
       </c>
       <c r="C19" s="18">
         <f>COUNTIF(Table_Tracker[Zone], B19)</f>
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="D19" s="18">
         <f>COUNTIFS(Table_Tracker[Zone], B19, Table_Tracker[Lock Type], "Planter")</f>
@@ -3312,7 +3318,7 @@
       </c>
       <c r="E19" s="18">
         <f>COUNTIFS(Table_Tracker[Zone], B19, Table_Tracker[Lock Type], "Cupboard")</f>
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="F19" s="18">
         <f>COUNTIFS(Table_Tracker[Zone], B19, Table_Tracker[Lock Type], "Locker")</f>
@@ -3344,7 +3350,7 @@
       </c>
       <c r="N19" s="5">
         <f>SUMIFS(Table_Tracker[Spare Keys (BMS)], Table_Tracker[Lock Type], "Door")</f>
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="O19" s="5">
         <f>SUMIFS(Table_Tracker[Issued Keys], Table_Tracker[Lock Type], "Door")</f>
@@ -3352,7 +3358,7 @@
       </c>
       <c r="P19" s="5">
         <f>SUMIFS(Table_Tracker[Missing Keys], Table_Tracker[Lock Type], "Door")</f>
-        <v>19</v>
+        <v>18</v>
       </c>
     </row>
     <row r="20" spans="2:16" ht="18" customHeight="1">
@@ -3401,7 +3407,7 @@
       </c>
       <c r="N20" s="5">
         <f>SUMIFS(Table_Tracker[Spare Keys (BMS)], Table_Tracker[Lock Type], "Locker")</f>
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="O20" s="5">
         <f>SUMIFS(Table_Tracker[Issued Keys], Table_Tracker[Lock Type], "Locker")</f>
@@ -3409,7 +3415,7 @@
       </c>
       <c r="P20" s="5">
         <f>SUMIFS(Table_Tracker[Missing Keys], Table_Tracker[Lock Type], "Locker")</f>
-        <v>11</v>
+        <v>10</v>
       </c>
     </row>
     <row r="21" spans="2:16" ht="18" customHeight="1">
@@ -3503,7 +3509,7 @@
       </c>
       <c r="K22" s="7">
         <f t="shared" ref="K22:P22" si="0">SUM(K17:K21)</f>
-        <v>243</v>
+        <v>244</v>
       </c>
       <c r="L22" s="7">
         <f t="shared" si="0"/>
@@ -3515,7 +3521,7 @@
       </c>
       <c r="N22" s="7">
         <f t="shared" si="0"/>
-        <v>372</v>
+        <v>376</v>
       </c>
       <c r="O22" s="7">
         <f t="shared" si="0"/>
@@ -3523,7 +3529,7 @@
       </c>
       <c r="P22" s="7">
         <f t="shared" si="0"/>
-        <v>68</v>
+        <v>66</v>
       </c>
     </row>
     <row r="23" spans="2:16" ht="18" customHeight="1">
@@ -3890,7 +3896,7 @@
       </c>
       <c r="C31" s="20">
         <f t="shared" ref="C31:H31" si="1">SUM(C17:C30)</f>
-        <v>244</v>
+        <v>245</v>
       </c>
       <c r="D31" s="20">
         <f t="shared" si="1"/>
@@ -3898,7 +3904,7 @@
       </c>
       <c r="E31" s="20">
         <f t="shared" si="1"/>
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="F31" s="20">
         <f t="shared" si="1"/>
@@ -13237,7 +13243,7 @@
         <v>✅ OK</v>
       </c>
     </row>
-    <row r="174" spans="1:16">
+    <row r="174" spans="1:16" hidden="1">
       <c r="A174" s="23">
         <v>167</v>
       </c>
@@ -13257,18 +13263,18 @@
         <v>2</v>
       </c>
       <c r="G174" s="23">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="H174" s="23">
         <v>0</v>
       </c>
       <c r="I174" s="23">
         <f t="shared" si="6"/>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J174" s="23" t="str">
         <f t="shared" si="7"/>
-        <v>⚠️ Missing Key</v>
+        <v>🔒 In Custody</v>
       </c>
       <c r="K174" s="23"/>
       <c r="L174" s="23" t="s">
@@ -13285,7 +13291,7 @@
       </c>
       <c r="P174" s="14" t="str">
         <f t="shared" si="8"/>
-        <v>🚨 REPLACE LOCK / KEY LOST</v>
+        <v>✅ OK</v>
       </c>
     </row>
     <row r="175" spans="1:16" hidden="1">
@@ -13484,7 +13490,9 @@
       <c r="L178" s="23" t="s">
         <v>63</v>
       </c>
-      <c r="M178" s="28"/>
+      <c r="M178" s="28" t="s">
+        <v>248</v>
+      </c>
       <c r="N178" s="14" t="s">
         <v>34</v>
       </c>
@@ -13846,9 +13854,11 @@
       <c r="L185" s="23" t="s">
         <v>233</v>
       </c>
-      <c r="M185" s="28"/>
+      <c r="M185" s="28" t="s">
+        <v>263</v>
+      </c>
       <c r="N185" s="14" t="s">
-        <v>263</v>
+        <v>264</v>
       </c>
       <c r="O185" s="14" t="s">
         <v>139</v>
@@ -13872,7 +13882,7 @@
         <v>31</v>
       </c>
       <c r="E186" s="23" t="s">
-        <v>264</v>
+        <v>265</v>
       </c>
       <c r="F186" s="23">
         <v>3</v>
@@ -13897,9 +13907,11 @@
       <c r="L186" s="23" t="s">
         <v>233</v>
       </c>
-      <c r="M186" s="28"/>
+      <c r="M186" s="28" t="s">
+        <v>263</v>
+      </c>
       <c r="N186" s="14" t="s">
-        <v>263</v>
+        <v>264</v>
       </c>
       <c r="O186" s="14" t="s">
         <v>139</v>
@@ -13923,7 +13935,7 @@
         <v>31</v>
       </c>
       <c r="E187" s="23" t="s">
-        <v>265</v>
+        <v>266</v>
       </c>
       <c r="F187" s="23">
         <v>3</v>
@@ -13948,9 +13960,11 @@
       <c r="L187" s="23" t="s">
         <v>233</v>
       </c>
-      <c r="M187" s="28"/>
+      <c r="M187" s="28" t="s">
+        <v>263</v>
+      </c>
       <c r="N187" s="14" t="s">
-        <v>263</v>
+        <v>264</v>
       </c>
       <c r="O187" s="14" t="s">
         <v>139</v>
@@ -13974,7 +13988,7 @@
         <v>31</v>
       </c>
       <c r="E188" s="23" t="s">
-        <v>266</v>
+        <v>267</v>
       </c>
       <c r="F188" s="23">
         <v>3</v>
@@ -13999,9 +14013,11 @@
       <c r="L188" s="23" t="s">
         <v>137</v>
       </c>
-      <c r="M188" s="28"/>
+      <c r="M188" s="28" t="s">
+        <v>263</v>
+      </c>
       <c r="N188" s="14" t="s">
-        <v>263</v>
+        <v>264</v>
       </c>
       <c r="O188" s="14" t="s">
         <v>139</v>
@@ -14025,7 +14041,7 @@
         <v>31</v>
       </c>
       <c r="E189" s="23" t="s">
-        <v>267</v>
+        <v>268</v>
       </c>
       <c r="F189" s="23">
         <v>3</v>
@@ -14050,9 +14066,11 @@
       <c r="L189" s="23" t="s">
         <v>137</v>
       </c>
-      <c r="M189" s="28"/>
+      <c r="M189" s="28" t="s">
+        <v>269</v>
+      </c>
       <c r="N189" s="14" t="s">
-        <v>263</v>
+        <v>264</v>
       </c>
       <c r="O189" s="14" t="s">
         <v>139</v>
@@ -14076,7 +14094,7 @@
         <v>31</v>
       </c>
       <c r="E190" s="23" t="s">
-        <v>268</v>
+        <v>270</v>
       </c>
       <c r="F190" s="23">
         <v>3</v>
@@ -14101,9 +14119,11 @@
       <c r="L190" s="23" t="s">
         <v>137</v>
       </c>
-      <c r="M190" s="28"/>
+      <c r="M190" s="28" t="s">
+        <v>263</v>
+      </c>
       <c r="N190" s="14" t="s">
-        <v>263</v>
+        <v>264</v>
       </c>
       <c r="O190" s="14" t="s">
         <v>139</v>
@@ -14127,7 +14147,7 @@
         <v>31</v>
       </c>
       <c r="E191" s="23" t="s">
-        <v>269</v>
+        <v>271</v>
       </c>
       <c r="F191" s="23">
         <v>3</v>
@@ -14152,9 +14172,11 @@
       <c r="L191" s="23" t="s">
         <v>137</v>
       </c>
-      <c r="M191" s="28"/>
+      <c r="M191" s="28" t="s">
+        <v>263</v>
+      </c>
       <c r="N191" s="14" t="s">
-        <v>263</v>
+        <v>264</v>
       </c>
       <c r="O191" s="14" t="s">
         <v>139</v>
@@ -14178,7 +14200,7 @@
         <v>31</v>
       </c>
       <c r="E192" s="23" t="s">
-        <v>270</v>
+        <v>272</v>
       </c>
       <c r="F192" s="23">
         <v>3</v>
@@ -14203,9 +14225,11 @@
       <c r="L192" s="23" t="s">
         <v>137</v>
       </c>
-      <c r="M192" s="28"/>
+      <c r="M192" s="28" t="s">
+        <v>263</v>
+      </c>
       <c r="N192" s="14" t="s">
-        <v>263</v>
+        <v>264</v>
       </c>
       <c r="O192" s="14" t="s">
         <v>139</v>
@@ -14229,7 +14253,7 @@
         <v>31</v>
       </c>
       <c r="E193" s="23" t="s">
-        <v>271</v>
+        <v>273</v>
       </c>
       <c r="F193" s="23">
         <v>3</v>
@@ -14254,9 +14278,11 @@
       <c r="L193" s="23" t="s">
         <v>137</v>
       </c>
-      <c r="M193" s="28"/>
+      <c r="M193" s="28" t="s">
+        <v>263</v>
+      </c>
       <c r="N193" s="14" t="s">
-        <v>263</v>
+        <v>264</v>
       </c>
       <c r="O193" s="14" t="s">
         <v>139</v>
@@ -14280,7 +14306,7 @@
         <v>31</v>
       </c>
       <c r="E194" s="23" t="s">
-        <v>272</v>
+        <v>274</v>
       </c>
       <c r="F194" s="23">
         <v>3</v>
@@ -14305,9 +14331,11 @@
       <c r="L194" s="23" t="s">
         <v>137</v>
       </c>
-      <c r="M194" s="28"/>
+      <c r="M194" s="28" t="s">
+        <v>263</v>
+      </c>
       <c r="N194" s="14" t="s">
-        <v>263</v>
+        <v>264</v>
       </c>
       <c r="O194" s="14" t="s">
         <v>139</v>
@@ -14331,7 +14359,7 @@
         <v>31</v>
       </c>
       <c r="E195" s="23" t="s">
-        <v>273</v>
+        <v>275</v>
       </c>
       <c r="F195" s="23">
         <v>3</v>
@@ -14356,9 +14384,11 @@
       <c r="L195" s="23" t="s">
         <v>137</v>
       </c>
-      <c r="M195" s="28"/>
+      <c r="M195" s="28" t="s">
+        <v>263</v>
+      </c>
       <c r="N195" s="14" t="s">
-        <v>263</v>
+        <v>264</v>
       </c>
       <c r="O195" s="14" t="s">
         <v>139</v>
@@ -14382,7 +14412,7 @@
         <v>31</v>
       </c>
       <c r="E196" s="23" t="s">
-        <v>274</v>
+        <v>276</v>
       </c>
       <c r="F196" s="23">
         <v>3</v>
@@ -14407,9 +14437,11 @@
       <c r="L196" s="23" t="s">
         <v>137</v>
       </c>
-      <c r="M196" s="28"/>
+      <c r="M196" s="28" t="s">
+        <v>263</v>
+      </c>
       <c r="N196" s="14" t="s">
-        <v>263</v>
+        <v>264</v>
       </c>
       <c r="O196" s="14" t="s">
         <v>139</v>
@@ -14433,7 +14465,7 @@
         <v>31</v>
       </c>
       <c r="E197" s="23" t="s">
-        <v>275</v>
+        <v>277</v>
       </c>
       <c r="F197" s="23">
         <v>3</v>
@@ -14458,9 +14490,11 @@
       <c r="L197" s="23" t="s">
         <v>137</v>
       </c>
-      <c r="M197" s="28"/>
+      <c r="M197" s="28" t="s">
+        <v>269</v>
+      </c>
       <c r="N197" s="14" t="s">
-        <v>263</v>
+        <v>264</v>
       </c>
       <c r="O197" s="14" t="s">
         <v>139</v>
@@ -14484,7 +14518,7 @@
         <v>31</v>
       </c>
       <c r="E198" s="23" t="s">
-        <v>276</v>
+        <v>278</v>
       </c>
       <c r="F198" s="23">
         <v>3</v>
@@ -14509,9 +14543,11 @@
       <c r="L198" s="23" t="s">
         <v>137</v>
       </c>
-      <c r="M198" s="28"/>
+      <c r="M198" s="28" t="s">
+        <v>263</v>
+      </c>
       <c r="N198" s="14" t="s">
-        <v>263</v>
+        <v>264</v>
       </c>
       <c r="O198" s="14" t="s">
         <v>139</v>
@@ -14535,7 +14571,7 @@
         <v>31</v>
       </c>
       <c r="E199" s="23" t="s">
-        <v>277</v>
+        <v>279</v>
       </c>
       <c r="F199" s="23">
         <v>3</v>
@@ -14560,9 +14596,11 @@
       <c r="L199" s="23" t="s">
         <v>137</v>
       </c>
-      <c r="M199" s="28"/>
+      <c r="M199" s="28" t="s">
+        <v>263</v>
+      </c>
       <c r="N199" s="14" t="s">
-        <v>263</v>
+        <v>264</v>
       </c>
       <c r="O199" s="14" t="s">
         <v>139</v>
@@ -14586,7 +14624,7 @@
         <v>31</v>
       </c>
       <c r="E200" s="23" t="s">
-        <v>278</v>
+        <v>280</v>
       </c>
       <c r="F200" s="23">
         <v>2</v>
@@ -14611,9 +14649,11 @@
       <c r="L200" s="23" t="s">
         <v>137</v>
       </c>
-      <c r="M200" s="28"/>
+      <c r="M200" s="28" t="s">
+        <v>263</v>
+      </c>
       <c r="N200" s="14" t="s">
-        <v>263</v>
+        <v>264</v>
       </c>
       <c r="O200" s="14" t="s">
         <v>139</v>
@@ -14637,7 +14677,7 @@
         <v>31</v>
       </c>
       <c r="E201" s="23" t="s">
-        <v>279</v>
+        <v>281</v>
       </c>
       <c r="F201" s="23">
         <v>3</v>
@@ -14662,9 +14702,11 @@
       <c r="L201" s="23" t="s">
         <v>137</v>
       </c>
-      <c r="M201" s="28"/>
+      <c r="M201" s="28" t="s">
+        <v>263</v>
+      </c>
       <c r="N201" s="14" t="s">
-        <v>263</v>
+        <v>264</v>
       </c>
       <c r="O201" s="14" t="s">
         <v>139</v>
@@ -14688,7 +14730,7 @@
         <v>31</v>
       </c>
       <c r="E202" s="23" t="s">
-        <v>280</v>
+        <v>282</v>
       </c>
       <c r="F202" s="23">
         <v>3</v>
@@ -14713,9 +14755,11 @@
       <c r="L202" s="23" t="s">
         <v>137</v>
       </c>
-      <c r="M202" s="28"/>
+      <c r="M202" s="28" t="s">
+        <v>263</v>
+      </c>
       <c r="N202" s="14" t="s">
-        <v>263</v>
+        <v>264</v>
       </c>
       <c r="O202" s="14" t="s">
         <v>139</v>
@@ -14739,7 +14783,7 @@
         <v>31</v>
       </c>
       <c r="E203" s="23" t="s">
-        <v>281</v>
+        <v>283</v>
       </c>
       <c r="F203" s="23">
         <v>3</v>
@@ -14764,9 +14808,11 @@
       <c r="L203" s="23" t="s">
         <v>137</v>
       </c>
-      <c r="M203" s="28"/>
+      <c r="M203" s="28" t="s">
+        <v>263</v>
+      </c>
       <c r="N203" s="14" t="s">
-        <v>263</v>
+        <v>264</v>
       </c>
       <c r="O203" s="14" t="s">
         <v>139</v>
@@ -14790,7 +14836,7 @@
         <v>31</v>
       </c>
       <c r="E204" s="23" t="s">
-        <v>282</v>
+        <v>284</v>
       </c>
       <c r="F204" s="23">
         <v>3</v>
@@ -14815,9 +14861,11 @@
       <c r="L204" s="23" t="s">
         <v>137</v>
       </c>
-      <c r="M204" s="28"/>
+      <c r="M204" s="28" t="s">
+        <v>263</v>
+      </c>
       <c r="N204" s="14" t="s">
-        <v>263</v>
+        <v>264</v>
       </c>
       <c r="O204" s="14" t="s">
         <v>139</v>
@@ -14841,7 +14889,7 @@
         <v>31</v>
       </c>
       <c r="E205" s="23" t="s">
-        <v>283</v>
+        <v>285</v>
       </c>
       <c r="F205" s="23">
         <v>3</v>
@@ -14866,9 +14914,11 @@
       <c r="L205" s="23" t="s">
         <v>137</v>
       </c>
-      <c r="M205" s="28"/>
+      <c r="M205" s="28" t="s">
+        <v>263</v>
+      </c>
       <c r="N205" s="14" t="s">
-        <v>263</v>
+        <v>264</v>
       </c>
       <c r="O205" s="14" t="s">
         <v>139</v>
@@ -14892,7 +14942,7 @@
         <v>31</v>
       </c>
       <c r="E206" s="23" t="s">
-        <v>284</v>
+        <v>286</v>
       </c>
       <c r="F206" s="23">
         <v>3</v>
@@ -14917,9 +14967,11 @@
       <c r="L206" s="23" t="s">
         <v>137</v>
       </c>
-      <c r="M206" s="28"/>
+      <c r="M206" s="28" t="s">
+        <v>263</v>
+      </c>
       <c r="N206" s="14" t="s">
-        <v>263</v>
+        <v>264</v>
       </c>
       <c r="O206" s="14" t="s">
         <v>139</v>
@@ -14943,24 +14995,24 @@
         <v>31</v>
       </c>
       <c r="E207" s="23" t="s">
-        <v>285</v>
+        <v>287</v>
       </c>
       <c r="F207" s="23">
         <v>3</v>
       </c>
       <c r="G207" s="23">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="H207" s="23">
         <v>0</v>
       </c>
       <c r="I207" s="23">
         <f t="shared" si="9"/>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J207" s="23" t="str">
         <f t="shared" si="10"/>
-        <v>⚠️ Missing Key</v>
+        <v>🔒 In Custody</v>
       </c>
       <c r="K207" s="23" t="s">
         <v>139</v>
@@ -14968,16 +15020,18 @@
       <c r="L207" s="23" t="s">
         <v>137</v>
       </c>
-      <c r="M207" s="28"/>
+      <c r="M207" s="28" t="s">
+        <v>263</v>
+      </c>
       <c r="N207" s="14" t="s">
-        <v>263</v>
+        <v>264</v>
       </c>
       <c r="O207" s="14" t="s">
         <v>139</v>
       </c>
       <c r="P207" s="14" t="str">
         <f t="shared" si="11"/>
-        <v>🚨 REPLACE LOCK / KEY LOST</v>
+        <v>✅ OK</v>
       </c>
     </row>
     <row r="208" spans="1:16" hidden="1">
@@ -14994,7 +15048,7 @@
         <v>31</v>
       </c>
       <c r="E208" s="23" t="s">
-        <v>286</v>
+        <v>288</v>
       </c>
       <c r="F208" s="23">
         <v>3</v>
@@ -15019,9 +15073,11 @@
       <c r="L208" s="23" t="s">
         <v>137</v>
       </c>
-      <c r="M208" s="28"/>
+      <c r="M208" s="28" t="s">
+        <v>263</v>
+      </c>
       <c r="N208" s="14" t="s">
-        <v>263</v>
+        <v>264</v>
       </c>
       <c r="O208" s="14" t="s">
         <v>139</v>
@@ -15045,7 +15101,7 @@
         <v>31</v>
       </c>
       <c r="E209" s="23" t="s">
-        <v>287</v>
+        <v>289</v>
       </c>
       <c r="F209" s="23">
         <v>3</v>
@@ -15070,9 +15126,11 @@
       <c r="L209" s="23" t="s">
         <v>137</v>
       </c>
-      <c r="M209" s="28"/>
+      <c r="M209" s="28" t="s">
+        <v>263</v>
+      </c>
       <c r="N209" s="14" t="s">
-        <v>263</v>
+        <v>264</v>
       </c>
       <c r="O209" s="14" t="s">
         <v>139</v>
@@ -15096,7 +15154,7 @@
         <v>31</v>
       </c>
       <c r="E210" s="23" t="s">
-        <v>288</v>
+        <v>290</v>
       </c>
       <c r="F210" s="23">
         <v>3</v>
@@ -15121,9 +15179,11 @@
       <c r="L210" s="23" t="s">
         <v>137</v>
       </c>
-      <c r="M210" s="28"/>
+      <c r="M210" s="28" t="s">
+        <v>263</v>
+      </c>
       <c r="N210" s="14" t="s">
-        <v>263</v>
+        <v>264</v>
       </c>
       <c r="O210" s="14" t="s">
         <v>139</v>
@@ -15147,7 +15207,7 @@
         <v>31</v>
       </c>
       <c r="E211" s="23" t="s">
-        <v>289</v>
+        <v>291</v>
       </c>
       <c r="F211" s="23">
         <v>3</v>
@@ -15172,9 +15232,11 @@
       <c r="L211" s="23" t="s">
         <v>137</v>
       </c>
-      <c r="M211" s="28"/>
+      <c r="M211" s="28" t="s">
+        <v>263</v>
+      </c>
       <c r="N211" s="14" t="s">
-        <v>263</v>
+        <v>264</v>
       </c>
       <c r="O211" s="14" t="s">
         <v>139</v>
@@ -15198,7 +15260,7 @@
         <v>31</v>
       </c>
       <c r="E212" s="23" t="s">
-        <v>290</v>
+        <v>292</v>
       </c>
       <c r="F212" s="23">
         <v>2</v>
@@ -15223,9 +15285,11 @@
       <c r="L212" s="23" t="s">
         <v>137</v>
       </c>
-      <c r="M212" s="28"/>
+      <c r="M212" s="28" t="s">
+        <v>263</v>
+      </c>
       <c r="N212" s="14" t="s">
-        <v>263</v>
+        <v>264</v>
       </c>
       <c r="O212" s="14" t="s">
         <v>139</v>
@@ -15235,7 +15299,7 @@
         <v>✅ OK</v>
       </c>
     </row>
-    <row r="213" spans="1:16" hidden="1">
+    <row r="213" spans="1:16">
       <c r="A213" s="23">
         <v>206</v>
       </c>
@@ -15300,7 +15364,7 @@
         <v>28</v>
       </c>
       <c r="E214" s="23" t="s">
-        <v>291</v>
+        <v>293</v>
       </c>
       <c r="F214" s="23">
         <v>2</v>
@@ -15320,7 +15384,7 @@
         <v>⚠️ Missing Key</v>
       </c>
       <c r="K214" s="23" t="s">
-        <v>292</v>
+        <v>294</v>
       </c>
       <c r="L214" s="23" t="s">
         <v>137</v>
@@ -15330,7 +15394,7 @@
         <v>34</v>
       </c>
       <c r="O214" s="14" t="s">
-        <v>293</v>
+        <v>295</v>
       </c>
       <c r="P214" s="14" t="str">
         <f t="shared" si="11"/>
@@ -15377,10 +15441,10 @@
         <v>137</v>
       </c>
       <c r="M215" s="28" t="s">
-        <v>294</v>
+        <v>296</v>
       </c>
       <c r="N215" s="14" t="s">
-        <v>263</v>
+        <v>264</v>
       </c>
       <c r="O215" s="14" t="s">
         <v>139</v>
@@ -15481,7 +15545,7 @@
         <v>137</v>
       </c>
       <c r="M217" s="28" t="s">
-        <v>295</v>
+        <v>297</v>
       </c>
       <c r="N217" s="14" t="s">
         <v>35</v>
@@ -15534,7 +15598,7 @@
         <v>137</v>
       </c>
       <c r="M218" s="28" t="s">
-        <v>296</v>
+        <v>298</v>
       </c>
       <c r="N218" s="14" t="s">
         <v>34</v>
@@ -15561,7 +15625,7 @@
         <v>28</v>
       </c>
       <c r="E219" s="23" t="s">
-        <v>297</v>
+        <v>299</v>
       </c>
       <c r="F219" s="23">
         <v>2</v>
@@ -15588,7 +15652,7 @@
       </c>
       <c r="M219" s="28"/>
       <c r="N219" s="14" t="s">
-        <v>263</v>
+        <v>264</v>
       </c>
       <c r="O219" s="14" t="s">
         <v>139</v>
@@ -15612,7 +15676,7 @@
         <v>31</v>
       </c>
       <c r="E220" s="23" t="s">
-        <v>298</v>
+        <v>300</v>
       </c>
       <c r="F220" s="23">
         <v>2</v>
@@ -15639,7 +15703,7 @@
       </c>
       <c r="M220" s="28"/>
       <c r="N220" s="14" t="s">
-        <v>263</v>
+        <v>264</v>
       </c>
       <c r="O220" s="14" t="s">
         <v>188</v>
@@ -15663,7 +15727,7 @@
         <v>31</v>
       </c>
       <c r="E221" s="23" t="s">
-        <v>299</v>
+        <v>301</v>
       </c>
       <c r="F221" s="23">
         <v>2</v>
@@ -15690,7 +15754,7 @@
       </c>
       <c r="M221" s="28"/>
       <c r="N221" s="14" t="s">
-        <v>263</v>
+        <v>264</v>
       </c>
       <c r="O221" s="14" t="s">
         <v>188</v>
@@ -15714,7 +15778,7 @@
         <v>31</v>
       </c>
       <c r="E222" s="23" t="s">
-        <v>300</v>
+        <v>302</v>
       </c>
       <c r="F222" s="23">
         <v>2</v>
@@ -15741,7 +15805,7 @@
       </c>
       <c r="M222" s="28"/>
       <c r="N222" s="14" t="s">
-        <v>263</v>
+        <v>264</v>
       </c>
       <c r="O222" s="14" t="s">
         <v>188</v>
@@ -15765,7 +15829,7 @@
         <v>31</v>
       </c>
       <c r="E223" s="23" t="s">
-        <v>301</v>
+        <v>303</v>
       </c>
       <c r="F223" s="23">
         <v>2</v>
@@ -15792,7 +15856,7 @@
       </c>
       <c r="M223" s="28"/>
       <c r="N223" s="14" t="s">
-        <v>263</v>
+        <v>264</v>
       </c>
       <c r="O223" s="14" t="s">
         <v>188</v>
@@ -15816,7 +15880,7 @@
         <v>31</v>
       </c>
       <c r="E224" s="23" t="s">
-        <v>302</v>
+        <v>304</v>
       </c>
       <c r="F224" s="23">
         <v>2</v>
@@ -15843,7 +15907,7 @@
       </c>
       <c r="M224" s="28"/>
       <c r="N224" s="14" t="s">
-        <v>263</v>
+        <v>264</v>
       </c>
       <c r="O224" s="14" t="s">
         <v>139</v>
@@ -15867,7 +15931,7 @@
         <v>31</v>
       </c>
       <c r="E225" s="23" t="s">
-        <v>303</v>
+        <v>305</v>
       </c>
       <c r="F225" s="23">
         <v>2</v>
@@ -15892,9 +15956,11 @@
       <c r="L225" s="23" t="s">
         <v>137</v>
       </c>
-      <c r="M225" s="28"/>
+      <c r="M225" s="28" t="s">
+        <v>263</v>
+      </c>
       <c r="N225" s="14" t="s">
-        <v>263</v>
+        <v>264</v>
       </c>
       <c r="O225" s="14" t="s">
         <v>139</v>
@@ -15918,7 +15984,7 @@
         <v>31</v>
       </c>
       <c r="E226" s="23" t="s">
-        <v>304</v>
+        <v>306</v>
       </c>
       <c r="F226" s="23">
         <v>3</v>
@@ -15943,9 +16009,11 @@
       <c r="L226" s="23" t="s">
         <v>137</v>
       </c>
-      <c r="M226" s="28"/>
+      <c r="M226" s="28" t="s">
+        <v>263</v>
+      </c>
       <c r="N226" s="14" t="s">
-        <v>263</v>
+        <v>264</v>
       </c>
       <c r="O226" s="14" t="s">
         <v>139</v>
@@ -15969,7 +16037,7 @@
         <v>31</v>
       </c>
       <c r="E227" s="23" t="s">
-        <v>305</v>
+        <v>307</v>
       </c>
       <c r="F227" s="23">
         <v>3</v>
@@ -15998,7 +16066,7 @@
         <v>177</v>
       </c>
       <c r="N227" s="14" t="s">
-        <v>263</v>
+        <v>264</v>
       </c>
       <c r="O227" s="14" t="s">
         <v>139</v>
@@ -16022,7 +16090,7 @@
         <v>31</v>
       </c>
       <c r="E228" s="23" t="s">
-        <v>306</v>
+        <v>308</v>
       </c>
       <c r="F228" s="23">
         <v>2</v>
@@ -16051,7 +16119,7 @@
         <v>177</v>
       </c>
       <c r="N228" s="14" t="s">
-        <v>263</v>
+        <v>264</v>
       </c>
       <c r="O228" s="14" t="s">
         <v>139</v>
@@ -16075,7 +16143,7 @@
         <v>31</v>
       </c>
       <c r="E229" s="23" t="s">
-        <v>307</v>
+        <v>309</v>
       </c>
       <c r="F229" s="23">
         <v>3</v>
@@ -16102,7 +16170,7 @@
       </c>
       <c r="M229" s="28"/>
       <c r="N229" s="14" t="s">
-        <v>263</v>
+        <v>264</v>
       </c>
       <c r="O229" s="14" t="s">
         <v>139</v>
@@ -16126,7 +16194,7 @@
         <v>31</v>
       </c>
       <c r="E230" s="23" t="s">
-        <v>308</v>
+        <v>310</v>
       </c>
       <c r="F230" s="23">
         <v>3</v>
@@ -16151,9 +16219,11 @@
       <c r="L230" s="23" t="s">
         <v>137</v>
       </c>
-      <c r="M230" s="28"/>
+      <c r="M230" s="28" t="s">
+        <v>263</v>
+      </c>
       <c r="N230" s="14" t="s">
-        <v>263</v>
+        <v>264</v>
       </c>
       <c r="O230" s="14" t="s">
         <v>139</v>
@@ -16177,7 +16247,7 @@
         <v>31</v>
       </c>
       <c r="E231" s="23" t="s">
-        <v>309</v>
+        <v>311</v>
       </c>
       <c r="F231" s="23">
         <v>3</v>
@@ -16202,9 +16272,11 @@
       <c r="L231" s="23" t="s">
         <v>233</v>
       </c>
-      <c r="M231" s="28"/>
+      <c r="M231" s="28" t="s">
+        <v>263</v>
+      </c>
       <c r="N231" s="14" t="s">
-        <v>263</v>
+        <v>264</v>
       </c>
       <c r="O231" s="14" t="s">
         <v>139</v>
@@ -16228,7 +16300,7 @@
         <v>31</v>
       </c>
       <c r="E232" s="23" t="s">
-        <v>310</v>
+        <v>312</v>
       </c>
       <c r="F232" s="23">
         <v>3</v>
@@ -16255,7 +16327,7 @@
       </c>
       <c r="M232" s="28"/>
       <c r="N232" s="14" t="s">
-        <v>263</v>
+        <v>264</v>
       </c>
       <c r="O232" s="14" t="s">
         <v>139</v>
@@ -16279,7 +16351,7 @@
         <v>31</v>
       </c>
       <c r="E233" s="23" t="s">
-        <v>311</v>
+        <v>313</v>
       </c>
       <c r="F233" s="23">
         <v>2</v>
@@ -16306,7 +16378,7 @@
       </c>
       <c r="M233" s="28"/>
       <c r="N233" s="14" t="s">
-        <v>263</v>
+        <v>264</v>
       </c>
       <c r="O233" s="14" t="s">
         <v>139</v>
@@ -16330,7 +16402,7 @@
         <v>31</v>
       </c>
       <c r="E234" s="23" t="s">
-        <v>312</v>
+        <v>314</v>
       </c>
       <c r="F234" s="23">
         <v>3</v>
@@ -16357,7 +16429,7 @@
       </c>
       <c r="M234" s="28"/>
       <c r="N234" s="14" t="s">
-        <v>263</v>
+        <v>264</v>
       </c>
       <c r="O234" s="14" t="s">
         <v>139</v>
@@ -16381,7 +16453,7 @@
         <v>31</v>
       </c>
       <c r="E235" s="23" t="s">
-        <v>313</v>
+        <v>315</v>
       </c>
       <c r="F235" s="23">
         <v>2</v>
@@ -16408,7 +16480,7 @@
       </c>
       <c r="M235" s="28"/>
       <c r="N235" s="14" t="s">
-        <v>263</v>
+        <v>264</v>
       </c>
       <c r="O235" s="14" t="s">
         <v>139</v>
@@ -16432,7 +16504,7 @@
         <v>31</v>
       </c>
       <c r="E236" s="23" t="s">
-        <v>314</v>
+        <v>316</v>
       </c>
       <c r="F236" s="23">
         <v>2</v>
@@ -16459,7 +16531,7 @@
       </c>
       <c r="M236" s="28"/>
       <c r="N236" s="14" t="s">
-        <v>263</v>
+        <v>264</v>
       </c>
       <c r="O236" s="14" t="s">
         <v>139</v>
@@ -16476,14 +16548,14 @@
       <c r="B237" s="23" t="s">
         <v>69</v>
       </c>
-      <c r="C237" s="26">
+      <c r="C237" s="24">
         <v>220</v>
       </c>
       <c r="D237" s="23" t="s">
         <v>31</v>
       </c>
       <c r="E237" s="23" t="s">
-        <v>315</v>
+        <v>317</v>
       </c>
       <c r="F237" s="23">
         <v>9</v>
@@ -16508,9 +16580,11 @@
       <c r="L237" s="23" t="s">
         <v>137</v>
       </c>
-      <c r="M237" s="28"/>
+      <c r="M237" s="28" t="s">
+        <v>263</v>
+      </c>
       <c r="N237" s="14" t="s">
-        <v>263</v>
+        <v>264</v>
       </c>
       <c r="O237" s="14" t="s">
         <v>139</v>
@@ -16534,7 +16608,7 @@
         <v>31</v>
       </c>
       <c r="E238" s="23" t="s">
-        <v>316</v>
+        <v>318</v>
       </c>
       <c r="F238" s="23">
         <v>4</v>
@@ -16561,7 +16635,7 @@
       </c>
       <c r="M238" s="28"/>
       <c r="N238" s="14" t="s">
-        <v>263</v>
+        <v>264</v>
       </c>
       <c r="O238" s="14" t="s">
         <v>139</v>
@@ -16585,7 +16659,7 @@
         <v>28</v>
       </c>
       <c r="E239" s="23" t="s">
-        <v>317</v>
+        <v>319</v>
       </c>
       <c r="F239" s="23">
         <v>2</v>
@@ -16608,14 +16682,14 @@
         <v>70</v>
       </c>
       <c r="L239" s="23" t="s">
-        <v>318</v>
+        <v>320</v>
       </c>
       <c r="M239" s="28"/>
       <c r="N239" s="14" t="s">
         <v>34</v>
       </c>
       <c r="O239" s="14" t="s">
-        <v>319</v>
+        <v>321</v>
       </c>
       <c r="P239" s="14" t="str">
         <f t="shared" si="11"/>
@@ -16636,7 +16710,7 @@
         <v>28</v>
       </c>
       <c r="E240" s="23" t="s">
-        <v>317</v>
+        <v>319</v>
       </c>
       <c r="F240" s="23">
         <v>2</v>
@@ -16659,14 +16733,14 @@
         <v>70</v>
       </c>
       <c r="L240" s="23" t="s">
-        <v>318</v>
+        <v>320</v>
       </c>
       <c r="M240" s="28"/>
       <c r="N240" s="14" t="s">
         <v>34</v>
       </c>
       <c r="O240" s="14" t="s">
-        <v>319</v>
+        <v>321</v>
       </c>
       <c r="P240" s="14" t="str">
         <f t="shared" si="11"/>
@@ -16687,7 +16761,7 @@
         <v>28</v>
       </c>
       <c r="E241" s="23" t="s">
-        <v>317</v>
+        <v>319</v>
       </c>
       <c r="F241" s="23">
         <v>2</v>
@@ -16710,14 +16784,14 @@
         <v>70</v>
       </c>
       <c r="L241" s="23" t="s">
-        <v>318</v>
+        <v>320</v>
       </c>
       <c r="M241" s="28"/>
       <c r="N241" s="14" t="s">
         <v>34</v>
       </c>
       <c r="O241" s="14" t="s">
-        <v>319</v>
+        <v>321</v>
       </c>
       <c r="P241" s="14" t="str">
         <f t="shared" si="11"/>
@@ -16738,7 +16812,7 @@
         <v>28</v>
       </c>
       <c r="E242" s="23" t="s">
-        <v>317</v>
+        <v>319</v>
       </c>
       <c r="F242" s="23">
         <v>2</v>
@@ -16761,14 +16835,14 @@
         <v>70</v>
       </c>
       <c r="L242" s="23" t="s">
-        <v>318</v>
+        <v>320</v>
       </c>
       <c r="M242" s="28"/>
       <c r="N242" s="14" t="s">
         <v>34</v>
       </c>
       <c r="O242" s="14" t="s">
-        <v>319</v>
+        <v>321</v>
       </c>
       <c r="P242" s="14" t="str">
         <f t="shared" si="11"/>
@@ -16789,7 +16863,7 @@
         <v>28</v>
       </c>
       <c r="E243" s="23" t="s">
-        <v>317</v>
+        <v>319</v>
       </c>
       <c r="F243" s="23">
         <v>2</v>
@@ -16812,14 +16886,14 @@
         <v>70</v>
       </c>
       <c r="L243" s="23" t="s">
-        <v>318</v>
+        <v>320</v>
       </c>
       <c r="M243" s="28"/>
       <c r="N243" s="14" t="s">
         <v>34</v>
       </c>
       <c r="O243" s="14" t="s">
-        <v>319</v>
+        <v>321</v>
       </c>
       <c r="P243" s="14" t="str">
         <f t="shared" si="11"/>
@@ -16840,7 +16914,7 @@
         <v>28</v>
       </c>
       <c r="E244" s="23" t="s">
-        <v>317</v>
+        <v>319</v>
       </c>
       <c r="F244" s="23">
         <v>2</v>
@@ -16863,14 +16937,14 @@
         <v>70</v>
       </c>
       <c r="L244" s="23" t="s">
-        <v>318</v>
+        <v>320</v>
       </c>
       <c r="M244" s="28"/>
       <c r="N244" s="14" t="s">
         <v>34</v>
       </c>
       <c r="O244" s="14" t="s">
-        <v>319</v>
+        <v>321</v>
       </c>
       <c r="P244" s="14" t="str">
         <f t="shared" si="11"/>
@@ -16920,10 +16994,10 @@
         <v>195</v>
       </c>
       <c r="N245" s="14" t="s">
-        <v>263</v>
+        <v>264</v>
       </c>
       <c r="O245" s="14" t="s">
-        <v>320</v>
+        <v>322</v>
       </c>
       <c r="P245" s="14" t="str">
         <f t="shared" si="11"/>
@@ -16973,10 +17047,10 @@
         <v>192</v>
       </c>
       <c r="N246" s="14" t="s">
-        <v>263</v>
+        <v>264</v>
       </c>
       <c r="O246" s="14" t="s">
-        <v>320</v>
+        <v>322</v>
       </c>
       <c r="P246" s="14" t="str">
         <f t="shared" si="11"/>
@@ -17026,10 +17100,10 @@
         <v>204</v>
       </c>
       <c r="N247" s="14" t="s">
-        <v>263</v>
+        <v>264</v>
       </c>
       <c r="O247" s="14" t="s">
-        <v>320</v>
+        <v>322</v>
       </c>
       <c r="P247" s="14" t="str">
         <f t="shared" si="11"/>
@@ -17050,7 +17124,7 @@
         <v>28</v>
       </c>
       <c r="E248" s="23" t="s">
-        <v>321</v>
+        <v>323</v>
       </c>
       <c r="F248" s="23">
         <v>2</v>
@@ -17076,13 +17150,13 @@
         <v>137</v>
       </c>
       <c r="M248" s="28" t="s">
-        <v>296</v>
+        <v>298</v>
       </c>
       <c r="N248" s="14" t="s">
-        <v>263</v>
+        <v>264</v>
       </c>
       <c r="O248" s="14" t="s">
-        <v>319</v>
+        <v>321</v>
       </c>
       <c r="P248" s="14" t="str">
         <f t="shared" si="11"/>
@@ -17103,7 +17177,7 @@
         <v>28</v>
       </c>
       <c r="E249" s="23" t="s">
-        <v>321</v>
+        <v>323</v>
       </c>
       <c r="F249" s="23">
         <v>2</v>
@@ -17129,13 +17203,13 @@
         <v>137</v>
       </c>
       <c r="M249" s="28" t="s">
-        <v>296</v>
+        <v>298</v>
       </c>
       <c r="N249" s="14" t="s">
-        <v>263</v>
+        <v>264</v>
       </c>
       <c r="O249" s="14" t="s">
-        <v>319</v>
+        <v>321</v>
       </c>
       <c r="P249" s="14" t="str">
         <f t="shared" si="11"/>
@@ -17189,7 +17263,7 @@
         <v>27</v>
       </c>
       <c r="E251" s="23" t="s">
-        <v>322</v>
+        <v>324</v>
       </c>
       <c r="F251" s="23">
         <v>2</v>
@@ -17223,26 +17297,55 @@
       </c>
     </row>
     <row r="252" spans="1:16" hidden="1">
-      <c r="A252" s="23"/>
-      <c r="B252" s="23"/>
-      <c r="C252" s="24"/>
-      <c r="D252" s="23"/>
-      <c r="E252" s="23"/>
-      <c r="F252" s="23"/>
-      <c r="G252" s="23"/>
-      <c r="H252" s="23"/>
-      <c r="I252" s="23"/>
+      <c r="A252" s="23">
+        <v>241</v>
+      </c>
+      <c r="B252" s="23" t="s">
+        <v>43</v>
+      </c>
+      <c r="C252" s="24">
+        <v>5555</v>
+      </c>
+      <c r="D252" s="23" t="s">
+        <v>28</v>
+      </c>
+      <c r="E252" s="23" t="s">
+        <v>323</v>
+      </c>
+      <c r="F252" s="23">
+        <v>2</v>
+      </c>
+      <c r="G252" s="23">
+        <v>2</v>
+      </c>
+      <c r="H252" s="23">
+        <v>0</v>
+      </c>
+      <c r="I252" s="23">
+        <f t="shared" ref="I252" si="12">MAX(0, F252-G252-H252)</f>
+        <v>0</v>
+      </c>
       <c r="J252" s="23" t="str">
-        <f t="shared" si="10"/>
-        <v>⚪ Unregistered</v>
-      </c>
-      <c r="K252" s="23"/>
-      <c r="L252" s="23"/>
-      <c r="M252" s="28"/>
-      <c r="N252" s="14"/>
-      <c r="O252" s="14"/>
+        <f t="shared" ref="J252" si="13">IF(I252&gt;0, "⚠️ Missing Key", IF(H252&gt;0, "🔑 Issued to Staff", IF(G252&gt;0, "🔒 In Custody", IF(F252=0, "⚪ Unregistered", "🔍 Under Audit"))))</f>
+        <v>🔒 In Custody</v>
+      </c>
+      <c r="K252" s="23" t="s">
+        <v>139</v>
+      </c>
+      <c r="L252" s="23" t="s">
+        <v>137</v>
+      </c>
+      <c r="M252" s="28" t="s">
+        <v>298</v>
+      </c>
+      <c r="N252" s="14" t="s">
+        <v>264</v>
+      </c>
+      <c r="O252" s="14" t="s">
+        <v>321</v>
+      </c>
       <c r="P252" s="14" t="str">
-        <f t="shared" si="11"/>
+        <f t="shared" ref="P252" si="14">IF(I252&gt;0, "🚨 REPLACE LOCK / KEY LOST", IF(ISNUMBER(SEARCH("Audit", O252)), "⚠️ AUDIT WITH EMPLOYEE", IF(ISNUMBER(SEARCH("Damaged", O252)), "⚠️ KEY DAMAGED / REPLACE", IF(ISNUMBER(SEARCH("Verification", O252)), "🔍 KEY VERIFICATION", IF(N252="Vacant", "🟢 AVAILABLE", "✅ OK")))))</f>
         <v>✅ OK</v>
       </c>
     </row>
@@ -17654,7 +17757,7 @@
     </row>
     <row r="4" spans="1:12" ht="24.95" customHeight="1">
       <c r="A4" s="40" t="s">
-        <v>323</v>
+        <v>325</v>
       </c>
       <c r="B4" s="69"/>
       <c r="C4" s="69"/>
@@ -17670,7 +17773,7 @@
     </row>
     <row r="5" spans="1:12" ht="18" customHeight="1">
       <c r="A5" s="54" t="s">
-        <v>324</v>
+        <v>326</v>
       </c>
       <c r="B5" s="69"/>
       <c r="C5" s="69"/>
@@ -17701,13 +17804,13 @@
         <v>124</v>
       </c>
       <c r="F7" s="15" t="s">
-        <v>325</v>
+        <v>327</v>
       </c>
       <c r="G7" s="15" t="s">
-        <v>326</v>
+        <v>328</v>
       </c>
       <c r="H7" s="15" t="s">
-        <v>327</v>
+        <v>329</v>
       </c>
       <c r="I7" s="15" t="s">
         <v>88</v>
@@ -17716,10 +17819,10 @@
         <v>89</v>
       </c>
       <c r="K7" s="15" t="s">
-        <v>328</v>
+        <v>330</v>
       </c>
       <c r="L7" s="15" t="s">
-        <v>329</v>
+        <v>331</v>
       </c>
     </row>
     <row r="8" spans="1:12">
@@ -17742,10 +17845,10 @@
         <v>188</v>
       </c>
       <c r="G8" s="23" t="s">
-        <v>330</v>
+        <v>332</v>
       </c>
       <c r="H8" s="23" t="s">
-        <v>331</v>
+        <v>333</v>
       </c>
       <c r="I8" s="23" t="s">
         <v>108</v>
@@ -17754,10 +17857,10 @@
         <v>109</v>
       </c>
       <c r="K8" s="23" t="s">
-        <v>332</v>
+        <v>334</v>
       </c>
       <c r="L8" s="23" t="s">
-        <v>333</v>
+        <v>335</v>
       </c>
     </row>
     <row r="9" spans="1:12">
@@ -17780,10 +17883,10 @@
         <v>188</v>
       </c>
       <c r="G9" s="23" t="s">
-        <v>330</v>
+        <v>332</v>
       </c>
       <c r="H9" s="23" t="s">
-        <v>331</v>
+        <v>333</v>
       </c>
       <c r="I9" s="23" t="s">
         <v>108</v>
@@ -17792,10 +17895,10 @@
         <v>109</v>
       </c>
       <c r="K9" s="23" t="s">
-        <v>332</v>
+        <v>334</v>
       </c>
       <c r="L9" s="23" t="s">
-        <v>334</v>
+        <v>336</v>
       </c>
     </row>
     <row r="10" spans="1:12">
@@ -17818,10 +17921,10 @@
         <v>188</v>
       </c>
       <c r="G10" s="23" t="s">
-        <v>330</v>
+        <v>332</v>
       </c>
       <c r="H10" s="23" t="s">
-        <v>331</v>
+        <v>333</v>
       </c>
       <c r="I10" s="23" t="s">
         <v>108</v>
@@ -17830,10 +17933,10 @@
         <v>109</v>
       </c>
       <c r="K10" s="23" t="s">
-        <v>332</v>
+        <v>334</v>
       </c>
       <c r="L10" s="23" t="s">
-        <v>335</v>
+        <v>337</v>
       </c>
     </row>
     <row r="11" spans="1:12">
@@ -17856,10 +17959,10 @@
         <v>198</v>
       </c>
       <c r="G11" s="23" t="s">
-        <v>336</v>
+        <v>338</v>
       </c>
       <c r="H11" s="23" t="s">
-        <v>337</v>
+        <v>339</v>
       </c>
       <c r="I11" s="23" t="s">
         <v>94</v>
@@ -17868,10 +17971,10 @@
         <v>95</v>
       </c>
       <c r="K11" s="23" t="s">
-        <v>332</v>
+        <v>334</v>
       </c>
       <c r="L11" s="23" t="s">
-        <v>338</v>
+        <v>340</v>
       </c>
     </row>
     <row r="12" spans="1:12">
@@ -17894,10 +17997,10 @@
         <v>188</v>
       </c>
       <c r="G12" s="23" t="s">
-        <v>330</v>
+        <v>332</v>
       </c>
       <c r="H12" s="23" t="s">
-        <v>331</v>
+        <v>333</v>
       </c>
       <c r="I12" s="23" t="s">
         <v>108</v>
@@ -17906,10 +18009,10 @@
         <v>109</v>
       </c>
       <c r="K12" s="23" t="s">
-        <v>332</v>
+        <v>334</v>
       </c>
       <c r="L12" s="23" t="s">
-        <v>339</v>
+        <v>341</v>
       </c>
     </row>
     <row r="13" spans="1:12">
@@ -17932,10 +18035,10 @@
         <v>201</v>
       </c>
       <c r="G13" s="23" t="s">
-        <v>330</v>
+        <v>332</v>
       </c>
       <c r="H13" s="23" t="s">
-        <v>331</v>
+        <v>333</v>
       </c>
       <c r="I13" s="23" t="s">
         <v>108</v>
@@ -17944,10 +18047,10 @@
         <v>109</v>
       </c>
       <c r="K13" s="23" t="s">
-        <v>332</v>
+        <v>334</v>
       </c>
       <c r="L13" s="23" t="s">
-        <v>340</v>
+        <v>342</v>
       </c>
     </row>
     <row r="14" spans="1:12">
@@ -17970,10 +18073,10 @@
         <v>188</v>
       </c>
       <c r="G14" s="23" t="s">
-        <v>330</v>
+        <v>332</v>
       </c>
       <c r="H14" s="23" t="s">
-        <v>331</v>
+        <v>333</v>
       </c>
       <c r="I14" s="23" t="s">
         <v>108</v>
@@ -17982,15 +18085,15 @@
         <v>109</v>
       </c>
       <c r="K14" s="23" t="s">
-        <v>332</v>
+        <v>334</v>
       </c>
       <c r="L14" s="23" t="s">
-        <v>341</v>
+        <v>343</v>
       </c>
     </row>
     <row r="15" spans="1:12">
       <c r="A15" s="23" t="s">
-        <v>342</v>
+        <v>344</v>
       </c>
       <c r="B15" s="23" t="s">
         <v>49</v>
@@ -18008,10 +18111,10 @@
         <v>188</v>
       </c>
       <c r="G15" s="23" t="s">
-        <v>330</v>
+        <v>332</v>
       </c>
       <c r="H15" s="23" t="s">
-        <v>331</v>
+        <v>333</v>
       </c>
       <c r="I15" s="23" t="s">
         <v>108</v>
@@ -18020,15 +18123,15 @@
         <v>109</v>
       </c>
       <c r="K15" s="23" t="s">
-        <v>332</v>
+        <v>334</v>
       </c>
       <c r="L15" s="23" t="s">
-        <v>343</v>
+        <v>345</v>
       </c>
     </row>
     <row r="16" spans="1:12">
       <c r="A16" s="23" t="s">
-        <v>344</v>
+        <v>346</v>
       </c>
       <c r="B16" s="23" t="s">
         <v>49</v>
@@ -18046,10 +18149,10 @@
         <v>188</v>
       </c>
       <c r="G16" s="23" t="s">
-        <v>330</v>
+        <v>332</v>
       </c>
       <c r="H16" s="23" t="s">
-        <v>331</v>
+        <v>333</v>
       </c>
       <c r="I16" s="23" t="s">
         <v>108</v>
@@ -18058,15 +18161,15 @@
         <v>109</v>
       </c>
       <c r="K16" s="23" t="s">
-        <v>332</v>
+        <v>334</v>
       </c>
       <c r="L16" s="23" t="s">
-        <v>345</v>
+        <v>347</v>
       </c>
     </row>
     <row r="17" spans="1:12">
       <c r="A17" s="23" t="s">
-        <v>346</v>
+        <v>348</v>
       </c>
       <c r="B17" s="23" t="s">
         <v>59</v>
@@ -18084,10 +18187,10 @@
         <v>234</v>
       </c>
       <c r="G17" s="23" t="s">
-        <v>330</v>
+        <v>332</v>
       </c>
       <c r="H17" s="23" t="s">
-        <v>331</v>
+        <v>333</v>
       </c>
       <c r="I17" s="23" t="s">
         <v>108</v>
@@ -18096,15 +18199,15 @@
         <v>109</v>
       </c>
       <c r="K17" s="23" t="s">
-        <v>332</v>
+        <v>334</v>
       </c>
       <c r="L17" s="23" t="s">
-        <v>347</v>
+        <v>349</v>
       </c>
     </row>
     <row r="18" spans="1:12">
       <c r="A18" s="23" t="s">
-        <v>348</v>
+        <v>350</v>
       </c>
       <c r="B18" s="23" t="s">
         <v>63</v>
@@ -18122,10 +18225,10 @@
         <v>237</v>
       </c>
       <c r="G18" s="23" t="s">
-        <v>330</v>
+        <v>332</v>
       </c>
       <c r="H18" s="23" t="s">
-        <v>331</v>
+        <v>333</v>
       </c>
       <c r="I18" s="23" t="s">
         <v>108</v>
@@ -18134,15 +18237,15 @@
         <v>109</v>
       </c>
       <c r="K18" s="23" t="s">
-        <v>332</v>
+        <v>334</v>
       </c>
       <c r="L18" s="23" t="s">
-        <v>349</v>
+        <v>351</v>
       </c>
     </row>
     <row r="19" spans="1:12">
       <c r="A19" s="23" t="s">
-        <v>350</v>
+        <v>352</v>
       </c>
       <c r="B19" s="23" t="s">
         <v>63</v>
@@ -18160,10 +18263,10 @@
         <v>237</v>
       </c>
       <c r="G19" s="23" t="s">
-        <v>330</v>
+        <v>332</v>
       </c>
       <c r="H19" s="23" t="s">
-        <v>331</v>
+        <v>333</v>
       </c>
       <c r="I19" s="23" t="s">
         <v>108</v>
@@ -18172,15 +18275,15 @@
         <v>109</v>
       </c>
       <c r="K19" s="23" t="s">
-        <v>332</v>
+        <v>334</v>
       </c>
       <c r="L19" s="23" t="s">
-        <v>351</v>
+        <v>353</v>
       </c>
     </row>
     <row r="20" spans="1:12">
       <c r="A20" s="23" t="s">
-        <v>352</v>
+        <v>354</v>
       </c>
       <c r="B20" s="23" t="s">
         <v>43</v>
@@ -18195,13 +18298,13 @@
         <v>103</v>
       </c>
       <c r="F20" s="27" t="s">
-        <v>353</v>
+        <v>355</v>
       </c>
       <c r="G20" s="23" t="s">
-        <v>336</v>
+        <v>338</v>
       </c>
       <c r="H20" s="23" t="s">
-        <v>337</v>
+        <v>339</v>
       </c>
       <c r="I20" s="23" t="s">
         <v>94</v>
@@ -18210,15 +18313,15 @@
         <v>95</v>
       </c>
       <c r="K20" s="23" t="s">
-        <v>332</v>
+        <v>334</v>
       </c>
       <c r="L20" s="23" t="s">
-        <v>354</v>
+        <v>356</v>
       </c>
     </row>
     <row r="21" spans="1:12">
       <c r="A21" s="23" t="s">
-        <v>355</v>
+        <v>357</v>
       </c>
       <c r="B21" s="23" t="s">
         <v>54</v>
@@ -18230,16 +18333,16 @@
         <v>31</v>
       </c>
       <c r="E21" s="23" t="s">
-        <v>298</v>
+        <v>300</v>
       </c>
       <c r="F21" s="27" t="s">
         <v>188</v>
       </c>
       <c r="G21" s="23" t="s">
-        <v>330</v>
+        <v>332</v>
       </c>
       <c r="H21" s="23" t="s">
-        <v>331</v>
+        <v>333</v>
       </c>
       <c r="I21" s="23" t="s">
         <v>108</v>
@@ -18248,15 +18351,15 @@
         <v>109</v>
       </c>
       <c r="K21" s="23" t="s">
-        <v>332</v>
+        <v>334</v>
       </c>
       <c r="L21" s="23" t="s">
-        <v>356</v>
+        <v>358</v>
       </c>
     </row>
     <row r="22" spans="1:12">
       <c r="A22" s="23" t="s">
-        <v>357</v>
+        <v>359</v>
       </c>
       <c r="B22" s="23" t="s">
         <v>45</v>
@@ -18268,16 +18371,16 @@
         <v>31</v>
       </c>
       <c r="E22" s="23" t="s">
-        <v>299</v>
+        <v>301</v>
       </c>
       <c r="F22" s="27" t="s">
         <v>188</v>
       </c>
       <c r="G22" s="23" t="s">
-        <v>330</v>
+        <v>332</v>
       </c>
       <c r="H22" s="23" t="s">
-        <v>331</v>
+        <v>333</v>
       </c>
       <c r="I22" s="23" t="s">
         <v>108</v>
@@ -18286,15 +18389,15 @@
         <v>109</v>
       </c>
       <c r="K22" s="23" t="s">
-        <v>332</v>
+        <v>334</v>
       </c>
       <c r="L22" s="23" t="s">
-        <v>358</v>
+        <v>360</v>
       </c>
     </row>
     <row r="23" spans="1:12">
       <c r="A23" s="23" t="s">
-        <v>359</v>
+        <v>361</v>
       </c>
       <c r="B23" s="23" t="s">
         <v>54</v>
@@ -18306,16 +18409,16 @@
         <v>31</v>
       </c>
       <c r="E23" s="23" t="s">
-        <v>300</v>
+        <v>302</v>
       </c>
       <c r="F23" s="27" t="s">
         <v>188</v>
       </c>
       <c r="G23" s="23" t="s">
-        <v>330</v>
+        <v>332</v>
       </c>
       <c r="H23" s="23" t="s">
-        <v>331</v>
+        <v>333</v>
       </c>
       <c r="I23" s="23" t="s">
         <v>108</v>
@@ -18324,15 +18427,15 @@
         <v>109</v>
       </c>
       <c r="K23" s="23" t="s">
-        <v>332</v>
+        <v>334</v>
       </c>
       <c r="L23" s="23" t="s">
-        <v>360</v>
+        <v>362</v>
       </c>
     </row>
     <row r="24" spans="1:12">
       <c r="A24" s="23" t="s">
-        <v>361</v>
+        <v>363</v>
       </c>
       <c r="B24" s="23" t="s">
         <v>54</v>
@@ -18344,16 +18447,16 @@
         <v>31</v>
       </c>
       <c r="E24" s="23" t="s">
-        <v>301</v>
+        <v>303</v>
       </c>
       <c r="F24" s="27" t="s">
         <v>188</v>
       </c>
       <c r="G24" s="23" t="s">
-        <v>330</v>
+        <v>332</v>
       </c>
       <c r="H24" s="23" t="s">
-        <v>331</v>
+        <v>333</v>
       </c>
       <c r="I24" s="23" t="s">
         <v>108</v>
@@ -18362,15 +18465,15 @@
         <v>109</v>
       </c>
       <c r="K24" s="23" t="s">
-        <v>332</v>
+        <v>334</v>
       </c>
       <c r="L24" s="23" t="s">
-        <v>362</v>
+        <v>364</v>
       </c>
     </row>
     <row r="25" spans="1:12" ht="29.1" customHeight="1">
       <c r="A25" s="23" t="s">
-        <v>363</v>
+        <v>365</v>
       </c>
       <c r="B25" s="23" t="s">
         <v>45</v>
@@ -18385,13 +18488,13 @@
         <v>92</v>
       </c>
       <c r="F25" s="27" t="s">
-        <v>320</v>
+        <v>322</v>
       </c>
       <c r="G25" s="23" t="s">
-        <v>336</v>
+        <v>338</v>
       </c>
       <c r="H25" s="23" t="s">
-        <v>337</v>
+        <v>339</v>
       </c>
       <c r="I25" s="23" t="s">
         <v>94</v>
@@ -18400,15 +18503,15 @@
         <v>95</v>
       </c>
       <c r="K25" s="23" t="s">
-        <v>332</v>
+        <v>334</v>
       </c>
       <c r="L25" s="23" t="s">
-        <v>364</v>
+        <v>366</v>
       </c>
     </row>
     <row r="26" spans="1:12" ht="29.1" customHeight="1">
       <c r="A26" s="23" t="s">
-        <v>365</v>
+        <v>367</v>
       </c>
       <c r="B26" s="23" t="s">
         <v>45</v>
@@ -18423,13 +18526,13 @@
         <v>92</v>
       </c>
       <c r="F26" s="27" t="s">
-        <v>320</v>
+        <v>322</v>
       </c>
       <c r="G26" s="23" t="s">
-        <v>336</v>
+        <v>338</v>
       </c>
       <c r="H26" s="23" t="s">
-        <v>337</v>
+        <v>339</v>
       </c>
       <c r="I26" s="23" t="s">
         <v>94</v>
@@ -18438,15 +18541,15 @@
         <v>95</v>
       </c>
       <c r="K26" s="23" t="s">
-        <v>332</v>
+        <v>334</v>
       </c>
       <c r="L26" s="23" t="s">
-        <v>366</v>
+        <v>368</v>
       </c>
     </row>
     <row r="27" spans="1:12" ht="29.1" customHeight="1">
       <c r="A27" s="23" t="s">
-        <v>367</v>
+        <v>369</v>
       </c>
       <c r="B27" s="23" t="s">
         <v>47</v>
@@ -18461,13 +18564,13 @@
         <v>100</v>
       </c>
       <c r="F27" s="27" t="s">
-        <v>320</v>
+        <v>322</v>
       </c>
       <c r="G27" s="23" t="s">
-        <v>336</v>
+        <v>338</v>
       </c>
       <c r="H27" s="23" t="s">
-        <v>337</v>
+        <v>339</v>
       </c>
       <c r="I27" s="23" t="s">
         <v>94</v>
@@ -18476,10 +18579,10 @@
         <v>95</v>
       </c>
       <c r="K27" s="23" t="s">
-        <v>332</v>
+        <v>334</v>
       </c>
       <c r="L27" s="23" t="s">
-        <v>368</v>
+        <v>370</v>
       </c>
     </row>
   </sheetData>
@@ -18563,7 +18666,7 @@
     </row>
     <row r="4" spans="2:14" ht="24.95" customHeight="1">
       <c r="B4" s="40" t="s">
-        <v>369</v>
+        <v>371</v>
       </c>
       <c r="C4" s="69"/>
       <c r="D4" s="69"/>
@@ -18580,7 +18683,7 @@
     </row>
     <row r="5" spans="2:14" ht="18" customHeight="1">
       <c r="B5" s="54" t="s">
-        <v>370</v>
+        <v>372</v>
       </c>
       <c r="C5" s="69"/>
       <c r="D5" s="69"/>
@@ -18597,7 +18700,7 @@
     </row>
     <row r="7" spans="2:14" ht="21.95" customHeight="1">
       <c r="B7" s="62" t="s">
-        <v>371</v>
+        <v>373</v>
       </c>
       <c r="C7" s="70"/>
       <c r="D7" s="70"/>
@@ -18614,25 +18717,25 @@
     </row>
     <row r="8" spans="2:14" ht="24" customHeight="1">
       <c r="B8" s="16" t="s">
-        <v>372</v>
+        <v>374</v>
       </c>
       <c r="C8" s="16" t="s">
         <v>26</v>
       </c>
       <c r="D8" s="16" t="s">
-        <v>373</v>
+        <v>375</v>
       </c>
       <c r="E8" s="16" t="s">
-        <v>374</v>
+        <v>376</v>
       </c>
       <c r="F8" s="16" t="s">
-        <v>375</v>
+        <v>377</v>
       </c>
       <c r="G8" s="16" t="s">
-        <v>376</v>
+        <v>378</v>
       </c>
       <c r="H8" s="16" t="s">
-        <v>377</v>
+        <v>379</v>
       </c>
       <c r="I8" s="16" t="s">
         <v>34</v>
@@ -18641,10 +18744,10 @@
         <v>35</v>
       </c>
       <c r="K8" s="16" t="s">
-        <v>378</v>
+        <v>380</v>
       </c>
       <c r="L8" s="16" t="s">
-        <v>379</v>
+        <v>381</v>
       </c>
       <c r="M8" s="16" t="s">
         <v>127</v>
@@ -18765,7 +18868,7 @@
       </c>
       <c r="C11" s="18">
         <f>COUNTIF(Table_Tracker[Zone], B11)</f>
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="D11" s="18">
         <f>COUNTIFS(Table_Tracker[Zone], B11, Table_Tracker[Lock Type], "Planter")</f>
@@ -18773,7 +18876,7 @@
       </c>
       <c r="E11" s="18">
         <f>COUNTIFS(Table_Tracker[Zone], B11, Table_Tracker[Lock Type], "Cupboard")</f>
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="F11" s="18">
         <f>COUNTIFS(Table_Tracker[Zone], B11, Table_Tracker[Lock Type], "Locker")</f>
@@ -18797,11 +18900,11 @@
       </c>
       <c r="K11" s="18">
         <f>COUNTIFS(Table_Tracker[Zone], B11, Table_Tracker[Lock Status], "Common Asset")</f>
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="L11" s="18">
         <f>SUMIFS(Table_Tracker[Spare Keys (BMS)], Table_Tracker[Zone], B11)</f>
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="M11" s="18">
         <f>SUMIFS(Table_Tracker[Issued Keys], Table_Tracker[Zone], B11)</f>
@@ -18960,7 +19063,7 @@
       </c>
       <c r="L14" s="18">
         <f>SUMIFS(Table_Tracker[Spare Keys (BMS)], Table_Tracker[Zone], B14)</f>
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="M14" s="18">
         <f>SUMIFS(Table_Tracker[Issued Keys], Table_Tracker[Zone], B14)</f>
@@ -18968,7 +19071,7 @@
       </c>
       <c r="N14" s="18">
         <f>SUMIFS(Table_Tracker[Missing Keys], Table_Tracker[Zone], B14)</f>
-        <v>17</v>
+        <v>16</v>
       </c>
     </row>
     <row r="15" spans="2:14" ht="18" customHeight="1">
@@ -19225,7 +19328,7 @@
       </c>
       <c r="L19" s="18">
         <f>SUMIFS(Table_Tracker[Spare Keys (BMS)], Table_Tracker[Zone], B19)</f>
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="M19" s="18">
         <f>SUMIFS(Table_Tracker[Issued Keys], Table_Tracker[Zone], B19)</f>
@@ -19233,7 +19336,7 @@
       </c>
       <c r="N19" s="18">
         <f>SUMIFS(Table_Tracker[Missing Keys], Table_Tracker[Zone], B19)</f>
-        <v>11</v>
+        <v>10</v>
       </c>
     </row>
     <row r="20" spans="2:14" ht="18" customHeight="1">
@@ -19397,11 +19500,11 @@
     </row>
     <row r="23" spans="2:14" ht="20.100000000000001" customHeight="1">
       <c r="B23" s="19" t="s">
-        <v>380</v>
+        <v>382</v>
       </c>
       <c r="C23" s="20">
         <f t="shared" ref="C23:N23" si="0">SUM(C9:C22)</f>
-        <v>244</v>
+        <v>245</v>
       </c>
       <c r="D23" s="20">
         <f t="shared" si="0"/>
@@ -19409,7 +19512,7 @@
       </c>
       <c r="E23" s="20">
         <f t="shared" si="0"/>
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="F23" s="20">
         <f t="shared" si="0"/>
@@ -19433,11 +19536,11 @@
       </c>
       <c r="K23" s="20">
         <f t="shared" si="0"/>
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="L23" s="20">
         <f t="shared" si="0"/>
-        <v>372</v>
+        <v>376</v>
       </c>
       <c r="M23" s="20">
         <f t="shared" si="0"/>
@@ -19445,7 +19548,7 @@
       </c>
       <c r="N23" s="20">
         <f t="shared" si="0"/>
-        <v>68</v>
+        <v>66</v>
       </c>
     </row>
   </sheetData>
@@ -19511,7 +19614,7 @@
     </row>
     <row r="4" spans="1:11" ht="24.95" customHeight="1">
       <c r="A4" s="40" t="s">
-        <v>381</v>
+        <v>383</v>
       </c>
       <c r="B4" s="69"/>
       <c r="C4" s="69"/>
@@ -19526,27 +19629,27 @@
     </row>
     <row r="5" spans="1:11" ht="15.95" customHeight="1">
       <c r="A5" s="3" t="s">
-        <v>382</v>
+        <v>384</v>
       </c>
       <c r="B5" s="15"/>
       <c r="C5" s="3" t="s">
-        <v>383</v>
+        <v>385</v>
       </c>
       <c r="D5" s="15"/>
       <c r="E5" s="3" t="s">
-        <v>384</v>
+        <v>386</v>
       </c>
       <c r="F5" s="15"/>
       <c r="G5" s="3" t="s">
-        <v>385</v>
+        <v>387</v>
       </c>
       <c r="H5" s="15"/>
       <c r="I5" s="3" t="s">
-        <v>386</v>
+        <v>388</v>
       </c>
       <c r="J5" s="15"/>
       <c r="K5" s="3" t="s">
-        <v>387</v>
+        <v>389</v>
       </c>
     </row>
     <row r="6" spans="1:11" ht="15.95" customHeight="1">
@@ -19571,7 +19674,7 @@
       </c>
       <c r="J6" s="15"/>
       <c r="K6" s="4" t="s">
-        <v>332</v>
+        <v>334</v>
       </c>
     </row>
     <row r="7" spans="1:11" ht="15.95" customHeight="1">
@@ -19596,7 +19699,7 @@
       </c>
       <c r="J7" s="15"/>
       <c r="K7" s="4" t="s">
-        <v>388</v>
+        <v>390</v>
       </c>
     </row>
     <row r="8" spans="1:11" ht="15.95" customHeight="1">
@@ -19609,19 +19712,19 @@
       </c>
       <c r="D8" s="15"/>
       <c r="E8" s="4" t="s">
-        <v>318</v>
+        <v>320</v>
       </c>
       <c r="F8" s="15"/>
       <c r="G8" s="4" t="s">
-        <v>263</v>
+        <v>264</v>
       </c>
       <c r="H8" s="15"/>
       <c r="I8" s="4" t="s">
-        <v>389</v>
+        <v>391</v>
       </c>
       <c r="J8" s="15"/>
       <c r="K8" s="4" t="s">
-        <v>390</v>
+        <v>392</v>
       </c>
     </row>
     <row r="9" spans="1:11" ht="15.95" customHeight="1">
@@ -19655,7 +19758,7 @@
       </c>
       <c r="D10" s="15"/>
       <c r="E10" s="4" t="s">
-        <v>391</v>
+        <v>393</v>
       </c>
       <c r="F10" s="15"/>
       <c r="G10" s="15"/>

</xml_diff>